<commit_message>
Repair error in design of special snapshots - they are now generated on the fly and not rely on historical data
</commit_message>
<xml_diff>
--- a/metrics_utility/test/snapshot_tests/CCSP/data/CCSP/snapshot_def_2024-02-01--2024-02-29/report.xlsx
+++ b/metrics_utility/test/snapshot_tests/CCSP/data/CCSP/snapshot_def_2024-02-01--2024-02-29/report.xlsx
@@ -523,7 +523,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>CCSP EU Direct Reporting Template</t>
+          <t>CCSP NA Direct Reporting Template</t>
         </is>
       </c>
     </row>
@@ -535,7 +535,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Partner B</t>
+          <t>Partner A</t>
         </is>
       </c>
     </row>
@@ -547,7 +547,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>support@partner.com</t>
+          <t>email@email.com</t>
         </is>
       </c>
     </row>
@@ -559,7 +559,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>admin_user</t>
+          <t>test_login</t>
         </is>
       </c>
     </row>
@@ -583,7 +583,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>DIRECTOR</t>
+          <t>BUSINESS LEADER</t>
         </is>
       </c>
     </row>
@@ -595,7 +595,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>PURCHASING HEAD</t>
+          <t>PROCUREMENT LEADER</t>
         </is>
       </c>
     </row>
@@ -663,12 +663,12 @@
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>CSP8794CE</t>
+          <t>MCT3752MO</t>
         </is>
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>EX: Red Hat OpenShift Container Platform, Premium Support (1 Node, Monthly)</t>
+          <t>EX: Red Hat Ansible Automation Platform, Full Support (1 Managed Node, Dedicated, Monthly)</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr"/>
@@ -689,7 +689,7 @@
       </c>
       <c r="G15" s="7" t="inlineStr">
         <is>
-          <t>15.01</t>
+          <t>11.55</t>
         </is>
       </c>
     </row>
@@ -736,7 +736,7 @@
         <v>1</v>
       </c>
       <c r="D18" s="10" t="n">
-        <v>15.01</v>
+        <v>11.55</v>
       </c>
       <c r="E18" s="10">
         <f>C18*D18</f>
@@ -754,7 +754,7 @@
         <v>2</v>
       </c>
       <c r="D19" s="10" t="n">
-        <v>15.01</v>
+        <v>11.55</v>
       </c>
       <c r="E19" s="10">
         <f>C19*D19</f>

</xml_diff>

<commit_message>
[AAP-87150] Default-enable indirect node report sheets and report type in metrics-utility (#559)
</commit_message>
<xml_diff>
--- a/metrics_utility/test/snapshot_tests/CCSP/data/CCSP/snapshot_def_2024-02-01--2024-02-29/report.xlsx
+++ b/metrics_utility/test/snapshot_tests/CCSP/data/CCSP/snapshot_def_2024-02-01--2024-02-29/report.xlsx
@@ -9,6 +9,10 @@
   <sheets>
     <sheet name="Usage Reporting" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Managed nodes" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Indirectly Managed nodes" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Usage by collections" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Usage by roles" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Usage by modules" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -84,7 +88,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="0000FF00"/>
+        <fgColor rgb="0092d050"/>
       </patternFill>
     </fill>
   </fills>
@@ -903,4 +907,248 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="25" customHeight="1">
+      <c r="A1" s="11" t="inlineStr">
+        <is>
+          <t>Host name</t>
+        </is>
+      </c>
+      <c r="B1" s="11" t="inlineStr">
+        <is>
+          <t>Automated by
+organizations</t>
+        </is>
+      </c>
+      <c r="C1" s="11" t="inlineStr">
+        <is>
+          <t>Job runs</t>
+        </is>
+      </c>
+      <c r="D1" s="11" t="inlineStr">
+        <is>
+          <t>Number of task
+runs</t>
+        </is>
+      </c>
+      <c r="E1" s="11" t="inlineStr">
+        <is>
+          <t>First
+automation</t>
+        </is>
+      </c>
+      <c r="F1" s="11" t="inlineStr">
+        <is>
+          <t>Last
+automation</t>
+        </is>
+      </c>
+      <c r="G1" s="11" t="inlineStr">
+        <is>
+          <t>Canonical
+Facts</t>
+        </is>
+      </c>
+      <c r="H1" s="11" t="inlineStr">
+        <is>
+          <t>Facts</t>
+        </is>
+      </c>
+      <c r="I1" s="11" t="inlineStr">
+        <is>
+          <t>Manage
+Node
+Types</t>
+        </is>
+      </c>
+      <c r="J1" s="11" t="inlineStr">
+        <is>
+          <t>Events</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="25" customHeight="1">
+      <c r="A1" s="11" t="inlineStr">
+        <is>
+          <t>Collection name</t>
+        </is>
+      </c>
+      <c r="B1" s="11" t="inlineStr">
+        <is>
+          <t>Unique managed nodes
+automated</t>
+        </is>
+      </c>
+      <c r="C1" s="11" t="inlineStr">
+        <is>
+          <t>Non-unique managed
+nodes automated</t>
+        </is>
+      </c>
+      <c r="D1" s="11" t="inlineStr">
+        <is>
+          <t>Number of task
+runs</t>
+        </is>
+      </c>
+      <c r="E1" s="11" t="inlineStr">
+        <is>
+          <t>Duration of task
+runs [seconds]</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="25" customHeight="1">
+      <c r="A1" s="11" t="inlineStr">
+        <is>
+          <t>Role name</t>
+        </is>
+      </c>
+      <c r="B1" s="11" t="inlineStr">
+        <is>
+          <t>Unique managed nodes
+automated</t>
+        </is>
+      </c>
+      <c r="C1" s="11" t="inlineStr">
+        <is>
+          <t>Non-unique managed
+nodes automated</t>
+        </is>
+      </c>
+      <c r="D1" s="11" t="inlineStr">
+        <is>
+          <t>Number of task
+runs</t>
+        </is>
+      </c>
+      <c r="E1" s="11" t="inlineStr">
+        <is>
+          <t>Duration of task
+runs [seconds]</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="25" customHeight="1">
+      <c r="A1" s="11" t="inlineStr">
+        <is>
+          <t>Module name</t>
+        </is>
+      </c>
+      <c r="B1" s="11" t="inlineStr">
+        <is>
+          <t>Unique managed nodes
+automated</t>
+        </is>
+      </c>
+      <c r="C1" s="11" t="inlineStr">
+        <is>
+          <t>Non-unique managed
+nodes automated</t>
+        </is>
+      </c>
+      <c r="D1" s="11" t="inlineStr">
+        <is>
+          <t>Number of task
+runs</t>
+        </is>
+      </c>
+      <c r="E1" s="11" t="inlineStr">
+        <is>
+          <t>Duration of task
+runs [seconds]</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>